<commit_message>
agregar sistema de automatizacion
</commit_message>
<xml_diff>
--- a/resultados/consolidado_limpio.xlsx
+++ b/resultados/consolidado_limpio.xlsx
@@ -16,7 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -46,8 +49,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G64"/>
+  <dimension ref="A1:G72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2518,6 +2522,254 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" s="1" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Teclado</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Electronica</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>2</v>
+      </c>
+      <c r="E65" t="n">
+        <v>65000</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Sofia</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Falda</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>1</v>
+      </c>
+      <c r="E66" t="n">
+        <v>52000</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Juan</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Tarjeta</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="n">
+        <v>46260</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Audifonos</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Electronica</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>3</v>
+      </c>
+      <c r="E67" t="n">
+        <v>38000</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Sofia</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="1" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Chaqueta</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>1</v>
+      </c>
+      <c r="E68" t="n">
+        <v>120000</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Juan</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Tarjeta</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="1" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Electronica</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>1</v>
+      </c>
+      <c r="E69" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Carlos</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Camisa</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>3</v>
+      </c>
+      <c r="E70" t="n">
+        <v>45000</v>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Ana</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Tarjeta</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="1" t="n">
+        <v>46260</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Mouse</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Electronica</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>4</v>
+      </c>
+      <c r="E71" t="n">
+        <v>35000</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Diego</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="1" t="n">
+        <v>46261</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Pantalon</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>2</v>
+      </c>
+      <c r="E72" t="n">
+        <v>89000</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Ana</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Tarjeta</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>